<commit_message>
:recycle: refactor: simplificando menu de importacao
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/template-importacao.xlsx
+++ b/template-importacao.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lancamentos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importacao" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,17 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="2">
@@ -51,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,6 +444,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Observação</t>
         </is>
       </c>
@@ -457,72 +456,78 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Salário</t>
+          <t>Santander Crédito</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Contribuição para casa</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Despesa</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5000,00</t>
+          <t>390,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Pago</t>
+          <t>Não pago</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Recebido dia 5</t>
-        </is>
-      </c>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Freelance</t>
+          <t>Nubank</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Entrada</t>
+          <t>Despesa</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1200,00</t>
+          <t>866,00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Pago</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aluguel</t>
+          <t>Milbane</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aluguel</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -532,7 +537,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1500,00</t>
+          <t>2000,00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -542,19 +547,24 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Vence dia 10</t>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Dívida</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Conta de luz</t>
+          <t>Dina (Faxina)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Luz</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -564,7 +574,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>185,90</t>
+          <t>25,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -572,17 +582,26 @@
           <t>Não pago</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mercado</t>
+          <t>Redfox</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mercado</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -592,7 +611,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>650,00</t>
+          <t>79,90</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -602,19 +621,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Compras do mês</t>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Recorrente no cartão</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Jovens de Maria</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Internet</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -624,89 +648,775 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>99,90</t>
+          <t>15,00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pago</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Como usar este template</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1. Preencha a aba Lancamentos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2. Tipo: Entrada ou Despesa</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>3. Status: Pago, Reservado ou Não pago</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>4. Valor com vírgula (ex: 150,90)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>5. No app: Importar &gt; Planilha CSV ou Excel</t>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Religioso</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6. Lançamentos vão para o mês atual.</t>
+          <t>MEI</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>86,05</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Impostos</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>86,05</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Impostos</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Backup total: use JSON.</t>
+          <t>Unha</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>135,00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Cuidados pessoais</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cabelo</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Cuidados pessoais</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Condução</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Combustível</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>135,00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Internet Vivo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>100,00</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Contribuição Casa</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Contribuição para casa</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Moradia</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Convênio Médico</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>589,36</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Família</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cartão Atacadão</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Cartão de crédito</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>563,06</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Dízimo</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Religioso</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Dízimo</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>50,00</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Religioso</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Combustível</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Combustível</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>350,00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>71,28</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Telefonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Camiseta São Pedro (2ª Parcela)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>40,00</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Vestuário</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Multa</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>234,00</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Raimunda</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>1000,00</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Não pago</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Investimento</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1000,00</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Reservado</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Viagem</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Investimento</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Reservado</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Reserva de Emergência PJ</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Investimento</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>500,00</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Reservado</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Reserva de Emergência PF</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Investimento</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>650,00</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Reservado</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Caixinha Turbo PF (Casa)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Investimento</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1200,00</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Reservado</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Reserva</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
:sparkles: feat: cartoes Gabriel e Babi com itens colapsaveis
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/template-importacao.xlsx
+++ b/template-importacao.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importacao" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão de crédito Gabriel</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão de crédito Babi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão de crédito Gabriel</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">

</xml_diff>